<commit_message>
feat: llm integration add secure OpenAI-compatible LLM provider configuration
</commit_message>
<xml_diff>
--- a/uat/manual_uat_checklist.xlsx
+++ b/uat/manual_uat_checklist.xlsx
@@ -18,8 +18,9 @@
     <sheet name="Image Downloader" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Job Recovery" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="Security Checks" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Defects" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="User Sign-Off" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="LLM Providers" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Defects" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="User Sign-Off" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Instructions'!$A$1:$B$7</definedName>
@@ -33,8 +34,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'Image Downloader'!$A$1:$K$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'Job Recovery'!$A$1:$K$6</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="10" hidden="1">'Security Checks'!$A$1:$K$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'Defects'!$A$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'User Sign-Off'!$A$1:$K$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="11" hidden="1">'LLM Providers'!$A$1:$K$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="12" hidden="1">'Defects'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="13" hidden="1">'User Sign-Off'!$A$1:$K$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1219,6 +1221,1006 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="34" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="5" max="5"/>
+    <col width="52" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Test ID</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Module</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Preconditions</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Input/Test Data</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Steps</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>Expected Result</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Actual Result</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Evidence/Screenshot</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>Defect ID</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>LLM-001</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Provider page</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>App is private.</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>LLM Providers</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>Open the page.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Provider list/form load; API key field is masked and blank.</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>LLM-002</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Add provider</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI-compatible test endpoint available.</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>Name, protocol, base URL, session key</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>Save without testing.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Provider is UNVERIFIED and no key appears in the list or database.</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>LLM-003</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Discovery</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Provider supports model listing.</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>Saved provider</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>Fetch models, search, and select one.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Sorted unique IDs appear; none is selected or activated automatically.</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>LLM-004</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Manual model</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>Model listing is unsupported.</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>Exact documented model ID</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>Enter vision/text model IDs manually.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Manual IDs save; activation remains blocked until tests pass.</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>LLM-005</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Text test</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Valid model/key.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>BYO_LLM_OK diagnostic</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>Run Test Connection after accepting the charge warning.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Exact token, auth, model, latency, safe request ID/usage, and unavailable/configured cost are reported.</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>LLM-006</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Structured test</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>Text test passed.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Fixed two-field schema</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>Run Test Structured Output.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Native or JSON compatibility is recorded; wrong/extra/malformed output fails.</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>LLM-007</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Vision test</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Vision model configured.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Generated blue-square image</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Run Test Vision.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Square/blue structured diagnostic passes without customer data.</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>LLM-008</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Activation</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>Required tests passed.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Vision and catalog purposes</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Select purposes and Save and Activate.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Only selected compatible routes activate; replacement requires confirmation.</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>LLM-009</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Separate routes</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Two tested models/providers available.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>Vision route A, catalog route B</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Activate separately and run one Topwear SKU.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Each service uses its route; history has non-secret snapshots and no fallback.</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>LLM-010</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Stale tests</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Active route exists.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>Changed model/timeout/key</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Edit and save.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Tests become STALE, route deactivates, and cached work is not reused.</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>LLM-011</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Wrong key</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Provider saved.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>Deliberately invalid test key</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Run text test.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Sanitized authentication failure; key absent from UI, logs, history, and SQLite.</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr"/>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>LLM-012</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Unknown model</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Valid key.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Nonexistent model ID</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Run tests and try activation.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Unknown model is sanitized and activation is blocked.</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr"/>
+      <c r="J13" s="2" t="inlineStr"/>
+      <c r="K13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>LLM-013</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Text-only model</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Text-capable model available.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>Same model as vision route</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Pass text; fail/skip vision; try activation.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Catalog may activate after required tests; vision cannot.</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr"/>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="2" t="inlineStr"/>
+      <c r="K14" s="2" t="inlineStr"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>LLM-014</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Session restart</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>SESSION_ONLY configured.</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>Fake test key</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Restart app/server and reopen provider.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Key is unavailable and must be re-entered; it was never persisted.</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr"/>
+      <c r="J15" s="2" t="inlineStr"/>
+      <c r="K15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>LLM-015</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Environment secret</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Test environment variable configured server-side.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>Variable name only</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Save ENV_REFERENCE and test.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Only the variable name persists; resolved value is never displayed.</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr"/>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="2" t="inlineStr"/>
+      <c r="K16" s="2" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>LLM-016</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>Encrypted secret</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Master key configured; app remains private.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>Fake test key</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>Save ENCRYPTED_DATABASE, edit blank, clear explicitly.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>SQLite has ciphertext only; blank preserves; confirmed clear removes it.</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr"/>
+      <c r="J17" s="2" t="inlineStr"/>
+      <c r="K17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>LLM-017</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>Endpoint blocks</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>No request should reach blocked targets.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>HTTP, localhost, private, metadata, credential URL</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>Try saving each with secure defaults.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>Every unsafe endpoint is rejected; no TLS-disable control exists.</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr"/>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="2" t="inlineStr"/>
+      <c r="K18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>LLM-018</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Local development</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Both local flags and exact allowlist configured outside production.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Local test endpoint</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>Save/test, then remove a flag and retry.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>Works only with required explicit development settings and strong warning.</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr"/>
+      <c r="J19" s="2" t="inlineStr"/>
+      <c r="K19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>LLM-019</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>Failure classes</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Mock/development endpoint available.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>401, 403, 404, 429, timeout, TLS, malformed</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>Trigger benign test failures.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>Each category is sanitized; no raw body, stack trace, header, or key appears.</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr"/>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="2" t="inlineStr"/>
+      <c r="K20" s="2" t="inlineStr"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>LLM-020</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>Retirement</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Provider has historical job snapshot.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>Used provider</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>Delete/retire it.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>Provider is disabled/retired; history remains readable and non-secret.</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr"/>
+      <c r="J21" s="2" t="inlineStr"/>
+      <c r="K21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>LLM-021</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>Secret search</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Use only a fake key.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>Unique fake value</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>Search logs and SQLite bytes after tests/restart.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>Fake key is absent wherever persistence/logging is forbidden.</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr"/>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>LLM-022</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>Existing pages</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Provider checks complete.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>CMS, downloader, history</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>Run existing offline workflows.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>All Phase 1–8 behavior still works.</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>NOT STARTED</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr"/>
+      <c r="J23" s="2" t="inlineStr"/>
+      <c r="K23" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K23"/>
+  <conditionalFormatting sqref="H2:H1000">
+    <cfRule type="expression" priority="1" dxfId="0">
+      <formula>$H2="PASS"</formula>
+    </cfRule>
+    <cfRule type="expression" priority="2" dxfId="1">
+      <formula>$H2="FAIL"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <dataValidations count="1">
+    <dataValidation sqref="H2:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"NOT STARTED,PASS,FAIL,BLOCKED,NOT APPLICABLE"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1311,7 +2313,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>